<commit_message>
M3 Excel docs: update unit test plan (45 tests PASS), agile sprint log, defect tracker (4 defects CLOSED)
</commit_message>
<xml_diff>
--- a/AI_QRS_Agile_Documentation.xlsx
+++ b/AI_QRS_Agile_Documentation.xlsx
@@ -45,7 +45,7 @@
     <numFmt numFmtId="164" formatCode="[$-1009]d/mmm/yy;@"/>
     <numFmt numFmtId="165" formatCode="[$-409]d\-mmm\-yy"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <name val="Arial"/>
       <family val="0"/>
@@ -142,8 +142,11 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -202,8 +205,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BDD7EE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -330,6 +343,83 @@
         <color rgb="00666666"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00666666"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00666666"/>
+      </left>
+      <right style="thin">
+        <color rgb="00666666"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00666666"/>
+      </left>
+      <right style="thin">
+        <color rgb="00666666"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00666666"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00666666"/>
+      </right>
+      <top style="thin">
+        <color rgb="00666666"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00666666"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00666666"/>
+      </right>
+      <top style="thin">
+        <color rgb="00666666"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00666666"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
@@ -356,7 +446,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="143">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -805,6 +895,12 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1129,7 +1225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I76"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.0546875" defaultRowHeight="12.75" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="65" min="1" max="1"/>
@@ -2194,6 +2290,461 @@
       <c r="G60" s="68" t="n"/>
       <c r="H60" s="68" t="n"/>
       <c r="I60" s="68" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="137" t="inlineStr">
+        <is>
+          <t>--- Milestone 3 Sprint Summary ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="138" t="inlineStr">
+        <is>
+          <t>Sprint</t>
+        </is>
+      </c>
+      <c r="B63" s="138" t="inlineStr">
+        <is>
+          <t>User Story</t>
+        </is>
+      </c>
+      <c r="C63" s="138" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D63" s="138" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E63" s="138" t="inlineStr">
+        <is>
+          <t>Completed Date</t>
+        </is>
+      </c>
+      <c r="F63" s="138" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B64" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.1</t>
+        </is>
+      </c>
+      <c r="C64" s="139" t="inlineStr">
+        <is>
+          <t>Clarification Agent - detects ambiguous queries and asks targeted questions</t>
+        </is>
+      </c>
+      <c r="D64" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E64" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F64" s="139" t="inlineStr">
+        <is>
+          <t>10/10 unit tests pass. Handles pronouns, vague nouns, open-ended follow-ups.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B65" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.1</t>
+        </is>
+      </c>
+      <c r="C65" s="139" t="inlineStr">
+        <is>
+          <t>Clarification cycle - refine_query() merges original + user response</t>
+        </is>
+      </c>
+      <c r="D65" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E65" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F65" s="139" t="inlineStr">
+        <is>
+          <t>Pronoun substitution, what-are/how-does patterns implemented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B66" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.2</t>
+        </is>
+      </c>
+      <c r="C66" s="139" t="inlineStr">
+        <is>
+          <t>Conversation Memory Agent - per-session bounded history (max 10)</t>
+        </is>
+      </c>
+      <c r="D66" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E66" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F66" s="139" t="inlineStr">
+        <is>
+          <t>Session isolation, topic tracking, history bounded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B67" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.2</t>
+        </is>
+      </c>
+      <c r="C67" s="139" t="inlineStr">
+        <is>
+          <t>Pronoun resolution - resolve_references() using active_key_terms</t>
+        </is>
+      </c>
+      <c r="D67" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E67" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F67" s="139" t="inlineStr">
+        <is>
+          <t>Bug fix: priority changed from last_entities to active_key_terms. Avoids ACME/boilerplate substitution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B68" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.2</t>
+        </is>
+      </c>
+      <c r="C68" s="139" t="inlineStr">
+        <is>
+          <t>Topic continuation vs context switch detection</t>
+        </is>
+      </c>
+      <c r="D68" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E68" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F68" s="139" t="inlineStr">
+        <is>
+          <t>is_topic_continuation() uses key-term overlap. Empty context returned on switch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B69" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.2</t>
+        </is>
+      </c>
+      <c r="C69" s="139" t="inlineStr">
+        <is>
+          <t>Clarification state stored in memory per session</t>
+        </is>
+      </c>
+      <c r="D69" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E69" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F69" s="139" t="inlineStr">
+        <is>
+          <t>set_clarification_pending/consume_clarification lifecycle working.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B70" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.3</t>
+        </is>
+      </c>
+      <c r="C70" s="139" t="inlineStr">
+        <is>
+          <t>Voice I/O - Speech-to-Text via Web Speech API</t>
+        </is>
+      </c>
+      <c r="D70" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E70" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F70" s="139" t="inlineStr">
+        <is>
+          <t>Browser-only. Mic button, transcript, error handling implemented in frontend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B71" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.3</t>
+        </is>
+      </c>
+      <c r="C71" s="139" t="inlineStr">
+        <is>
+          <t>Voice I/O - Text-to-Speech for answer readback</t>
+        </is>
+      </c>
+      <c r="D71" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E71" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F71" s="139" t="inlineStr">
+        <is>
+          <t>TTS controls: play, pause, stop in frontend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B72" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.4</t>
+        </is>
+      </c>
+      <c r="C72" s="139" t="inlineStr">
+        <is>
+          <t>Transparency Panel - sources with text, page, chunk_id, score, citation</t>
+        </is>
+      </c>
+      <c r="D72" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E72" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F72" s="139" t="inlineStr">
+        <is>
+          <t>All 10 M3.4 fields present in every source dict. Text truncated at 600 chars.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B73" s="139" t="inlineStr">
+        <is>
+          <t>US-M3.4</t>
+        </is>
+      </c>
+      <c r="C73" s="139" t="inlineStr">
+        <is>
+          <t>Knowledge Gap handling - confidence=0, controlled response</t>
+        </is>
+      </c>
+      <c r="D73" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E73" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F73" s="139" t="inlineStr">
+        <is>
+          <t>No unsupported answers generated when retrieval returns empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B74" s="139" t="inlineStr">
+        <is>
+          <t>BUG-FIX</t>
+        </is>
+      </c>
+      <c r="C74" s="139" t="inlineStr">
+        <is>
+          <t>retrieval_agent: similarity_threshold default 0.0 -&gt; None</t>
+        </is>
+      </c>
+      <c r="D74" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E74" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F74" s="139" t="inlineStr">
+        <is>
+          <t>settings.similarity_threshold now honoured correctly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B75" s="139" t="inlineStr">
+        <is>
+          <t>BUG-FIX</t>
+        </is>
+      </c>
+      <c r="C75" s="139" t="inlineStr">
+        <is>
+          <t>orchestrator: UnboundLocalError resolved_query in clarification path</t>
+        </is>
+      </c>
+      <c r="D75" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E75" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F75" s="139" t="inlineStr">
+        <is>
+          <t>resolved_query always assigned: refined_query or memory_resolved_query.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="139" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="B76" s="139" t="inlineStr">
+        <is>
+          <t>BUG-FIX</t>
+        </is>
+      </c>
+      <c r="C76" s="139" t="inlineStr">
+        <is>
+          <t>retrieval_agent: pass resolved_query for vector search</t>
+        </is>
+      </c>
+      <c r="D76" s="139" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E76" s="139" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="F76" s="139" t="inlineStr">
+        <is>
+          <t>Pronoun-resolved text now used for embedding, not raw normalized query.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I11"/>
@@ -2395,14 +2946,14 @@
       </c>
     </row>
     <row r="3" ht="30" customHeight="1" s="65">
-      <c r="A3" s="124" t="n"/>
-      <c r="B3" s="125" t="n"/>
-      <c r="C3" s="126" t="n"/>
-      <c r="D3" s="126" t="n"/>
-      <c r="E3" s="126" t="n"/>
-      <c r="F3" s="126" t="n"/>
-      <c r="G3" s="126" t="n"/>
-      <c r="H3" s="126" t="n"/>
+      <c r="A3" s="140" t="n"/>
+      <c r="B3" s="140" t="n"/>
+      <c r="C3" s="140" t="n"/>
+      <c r="D3" s="140" t="n"/>
+      <c r="E3" s="140" t="n"/>
+      <c r="F3" s="140" t="n"/>
+      <c r="G3" s="140" t="n"/>
+      <c r="H3" s="140" t="n"/>
       <c r="I3" s="93">
         <f>SUM(I5:I802)</f>
         <v/>
@@ -2470,28 +3021,28 @@
           <t>SPRINT 1 BACKLOG</t>
         </is>
       </c>
-      <c r="B4" s="128" t="n"/>
-      <c r="C4" s="128" t="n"/>
-      <c r="D4" s="128" t="n"/>
-      <c r="E4" s="128" t="n"/>
-      <c r="F4" s="128" t="n"/>
-      <c r="G4" s="128" t="n"/>
-      <c r="H4" s="128" t="n"/>
-      <c r="I4" s="128" t="n"/>
-      <c r="J4" s="128" t="n"/>
-      <c r="K4" s="128" t="n"/>
-      <c r="L4" s="128" t="n"/>
-      <c r="M4" s="128" t="n"/>
-      <c r="N4" s="128" t="n"/>
-      <c r="O4" s="128" t="n"/>
-      <c r="P4" s="128" t="n"/>
-      <c r="Q4" s="128" t="n"/>
-      <c r="R4" s="128" t="n"/>
-      <c r="S4" s="128" t="n"/>
-      <c r="T4" s="128" t="n"/>
-      <c r="U4" s="128" t="n"/>
-      <c r="V4" s="128" t="n"/>
-      <c r="W4" s="129" t="n"/>
+      <c r="B4" s="141" t="n"/>
+      <c r="C4" s="141" t="n"/>
+      <c r="D4" s="141" t="n"/>
+      <c r="E4" s="141" t="n"/>
+      <c r="F4" s="141" t="n"/>
+      <c r="G4" s="141" t="n"/>
+      <c r="H4" s="141" t="n"/>
+      <c r="I4" s="141" t="n"/>
+      <c r="J4" s="141" t="n"/>
+      <c r="K4" s="141" t="n"/>
+      <c r="L4" s="141" t="n"/>
+      <c r="M4" s="141" t="n"/>
+      <c r="N4" s="141" t="n"/>
+      <c r="O4" s="141" t="n"/>
+      <c r="P4" s="141" t="n"/>
+      <c r="Q4" s="141" t="n"/>
+      <c r="R4" s="141" t="n"/>
+      <c r="S4" s="141" t="n"/>
+      <c r="T4" s="141" t="n"/>
+      <c r="U4" s="141" t="n"/>
+      <c r="V4" s="141" t="n"/>
+      <c r="W4" s="142" t="n"/>
     </row>
     <row r="5" ht="55" customHeight="1" s="65">
       <c r="A5" s="130" t="inlineStr">

</xml_diff>